<commit_message>
E1 live site 2026-09-16 23:56 IST
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/E1-BLOTTER.xlsx
+++ b/E1-BLOTTER.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="64">
   <si>
     <t>source</t>
   </si>
@@ -563,7 +563,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S17"/>
+  <dimension ref="A1:S16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:19">
@@ -1339,62 +1339,6 @@
         <v>63</v>
       </c>
     </row>
-    <row r="17" spans="1:19">
-      <c r="A17" t="s">
-        <v>21</v>
-      </c>
-      <c r="B17" t="s">
-        <v>23</v>
-      </c>
-      <c r="D17">
-        <v>1</v>
-      </c>
-      <c r="E17" t="s">
-        <v>43</v>
-      </c>
-      <c r="F17" t="s">
-        <v>44</v>
-      </c>
-      <c r="G17" t="s">
-        <v>56</v>
-      </c>
-      <c r="H17" t="s">
-        <v>57</v>
-      </c>
-      <c r="I17" t="s">
-        <v>58</v>
-      </c>
-      <c r="J17">
-        <v>100</v>
-      </c>
-      <c r="K17">
-        <v>99</v>
-      </c>
-      <c r="L17">
-        <v>101</v>
-      </c>
-      <c r="M17">
-        <v>99</v>
-      </c>
-      <c r="N17" t="s">
-        <v>60</v>
-      </c>
-      <c r="O17">
-        <v>-1</v>
-      </c>
-      <c r="P17">
-        <v>-1000</v>
-      </c>
-      <c r="Q17" t="s">
-        <v>62</v>
-      </c>
-      <c r="R17" t="s">
-        <v>23</v>
-      </c>
-      <c r="S17" t="s">
-        <v>63</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>